<commit_message>
Daily NSE scan: 2026-09-12
</commit_message>
<xml_diff>
--- a/output/2026-09-12/enriched_analysis.xlsx
+++ b/output/2026-09-12/enriched_analysis.xlsx
@@ -3670,7 +3670,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>INE577L01016</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -4398,7 +4398,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -8447,7 +8447,7 @@
         <v>-0.18</v>
       </c>
       <c r="X44" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="Y44" t="b">
         <v>0</v>
@@ -9536,10 +9536,10 @@
         <v>0.21</v>
       </c>
       <c r="W50" t="n">
-        <v>17.6</v>
+        <v>18</v>
       </c>
       <c r="X50" t="n">
-        <v>0.31</v>
+        <v>0.32</v>
       </c>
       <c r="Y50" t="b">
         <v>0</v>
@@ -10282,7 +10282,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>STEL HOLDINGS LIMITED</t>
+          <t>INE577L01016</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -10422,7 +10422,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>PNGS REVA DIAMOND JEWELLERY LIMITED</t>
+          <t>PNGS Reva Diamond Jewellery Limited</t>
         </is>
       </c>
       <c r="C22" t="n">

</xml_diff>